<commit_message>
🔧 FIX: Correct Table 1 to show Detection (Images) vs Classification (Boxes)
- Detection counts FULL IMAGES (fewer data points)
  * IML: 206/56/51 = 313 images
  * MP-IDB: 137/36/36 = 209 images
  * MD_2019: 1028/270/328 = 1626 images

- Classification counts BOUNDING BOX CROPS (more data points)
  * IML: 412/112/102 = 626 boxes (2.0× per image)
  * MP-IDB: 274/72/72 = 418 boxes (2.0× per image)
  * MD_2019: 1028/270/328 = 1626 boxes (1.0× per image)

- Updated Table 1 caption to clarify difference
- Backed up old table as Table1_Dataset_Augmentation_OLD_BACKUP.xlsx

Root cause: Split performed at IMAGE level, but detection counts images while
classification counts boxes/crops extracted from those images.
</commit_message>
<xml_diff>
--- a/luaran/templates/tables/Table1_Dataset_Augmentation.xlsx
+++ b/luaran/templates/tables/Table1_Dataset_Augmentation.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,7 +36,16 @@
       <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -54,14 +63,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="005B9BD5"/>
-        <bgColor rgb="005B9BD5"/>
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,26 +92,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,175 +477,152 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Detection Training (Full Images)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Classification Training (Cropped Bounding Boxes)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Original Data (60/20/20 Split)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Detection Training Data
-(4.4× Augmentation on Train Only)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Classification Training Data
-(3.5× Augmentation on Train Only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="25" customHeight="1">
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Train</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Val</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Train</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Val</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Train</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Val</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="35" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>IML Lifecycle
-(4 stages)</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Train (Images)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Val (Images)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Test (Images)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Total Images</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Train (Crops)</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Val (Crops)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Test (Crops)</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Total Crops</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Boxes per Image Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>IML Lifecycle (4 stages)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>206</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>313</v>
+      </c>
+      <c r="F3" s="5" t="n">
         <v>412</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>112</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="H3" s="5" t="n">
         <v>102</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="I3" s="5" t="n">
         <v>626</v>
       </c>
-      <c r="F3" s="4" t="n">
-        <v>1807</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>112</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>102</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>1446</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>112</v>
-      </c>
-      <c r="L3" s="4" t="n">
-        <v>102</v>
-      </c>
-      <c r="M3" s="4" t="n">
-        <v>1660</v>
-      </c>
-    </row>
-    <row r="4" ht="35" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>MP-IDB Species
-(4 species)</t>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>2.0×</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MP-IDB Species (4 species)</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
+        <v>137</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>209</v>
+      </c>
+      <c r="F4" s="6" t="n">
         <v>274</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>72</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>72</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>418</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>1202</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>72</v>
@@ -645,70 +631,54 @@
         <v>72</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>1346</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>961</v>
-      </c>
-      <c r="K4" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>2.0×</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>MP-IDB Stages (4 stages)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>209</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>274</v>
+      </c>
+      <c r="G5" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="L4" s="6" t="n">
+      <c r="H5" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="M4" s="6" t="n">
-        <v>1105</v>
-      </c>
-    </row>
-    <row r="5" ht="35" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>MP-IDB Stages
-(4 stages)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>274</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="E5" s="4" t="n">
+      <c r="I5" s="5" t="n">
         <v>418</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>1202</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>1346</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>961</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="M5" s="4" t="n">
-        <v>1105</v>
-      </c>
-    </row>
-    <row r="6" ht="35" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>MD_2019 Stages
-(3 stages)</t>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>2.0×</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MD_2019 Stages (3 stages)</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -724,7 +694,7 @@
         <v>1626</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>4510</v>
+        <v>1028</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>270</v>
@@ -733,27 +703,58 @@
         <v>328</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>5108</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>3608</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>270</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <v>328</v>
-      </c>
-      <c r="M6" s="6" t="n">
-        <v>4206</v>
+        <v>1626</v>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>1.0×</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Note:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>• Detection counts FULL IMAGES (one image = one data point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>• Classification counts BOUNDING BOX CROPS (one image can contain multiple boxes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>• Split performed at IMAGE level (60/20/20), then crops extracted → crop counts differ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>• Augmentation: Detection 4.4× on train only, Classification 3.5× on train only</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="A1:A2"/>
+  <mergeCells count="7">
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:J1"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="A11:J11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✨ COMPLETE: Add augmentation columns back to Table 1
Table 1 now shows COMPLETE picture:
1. Detection (Full Images) - before augmentation
   - IML: 206/56/51 = 313 images
   - MP-IDB: 137/36/36 = 209 images
   - MD_2019: 1028/270/328 = 1626 images

2. Classification (Bounding Box Crops) - before augmentation
   - IML: 412/112/102 = 626 boxes (2.0× per image)
   - MP-IDB: 274/72/72 = 418 boxes (2.0× per image)
   - MD_2019: 1028/270/328 = 1626 boxes (1.0× per image)

3. After Augmentation (Train Only)
   - Detection: 4.4× multiplier
   - Classification: 3.5× multiplier
   - Val and Test remain UNAUGMENTED

4. Boxes per Image ratio column

User feedback: Missing augmentation data columns
</commit_message>
<xml_diff>
--- a/luaran/templates/tables/Table1_Dataset_Augmentation.xlsx
+++ b/luaran/templates/tables/Table1_Dataset_Augmentation.xlsx
@@ -28,15 +28,16 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -92,8 +93,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -102,7 +106,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -477,284 +481,368 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Detection Training (Full Images)</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Classification Training (Cropped Bounding Boxes)</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Detection (Full Images)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="n"/>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Classification (Bounding Box Crops)</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="n"/>
+      <c r="I1" s="3" t="n"/>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>After Augmentation (Train Only)</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="n"/>
+      <c r="L1" s="3" t="n"/>
+      <c r="M1" s="3" t="n"/>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Boxes per Image</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Dataset</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Train (Images)</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Val (Images)</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Test (Images)</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Total Images</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Train (Crops)</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Val (Crops)</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Test (Crops)</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Total Crops</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Boxes per Image Ratio</t>
-        </is>
-      </c>
+      <c r="A2" s="3" t="n"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Train</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Val</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Train</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Val</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Det Train (4.4×)</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>Cls Train (3.5×)</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Val (same)</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>Test (same)</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>IML Lifecycle (4 stages)</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>IML Lifecycle
+(4 stages)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="6" t="n">
         <v>56</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="6" t="n">
         <v>313</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="6" t="n">
         <v>412</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="6" t="n">
         <v>112</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="6" t="n">
         <v>102</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="I3" s="6" t="n">
         <v>626</v>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="6" t="n">
+        <v>906</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>1442</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="M3" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>2.0×</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>MP-IDB Species (4 species)</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>MP-IDB Species
+(4 species)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
         <v>137</v>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="7" t="n">
         <v>209</v>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="7" t="n">
         <v>274</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="7" t="n">
         <v>72</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="7" t="n">
         <v>72</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="7" t="n">
         <v>418</v>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="7" t="n">
+        <v>602</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>959</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>2.0×</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>MP-IDB Stages (4 stages)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>MP-IDB Stages
+(4 stages)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
         <v>137</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="6" t="n">
         <v>209</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="6" t="n">
         <v>274</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="6" t="n">
         <v>72</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="6" t="n">
         <v>72</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="6" t="n">
         <v>418</v>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="6" t="n">
+        <v>602</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>959</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>2.0×</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>MD_2019 Stages (3 stages)</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>MD_2019 Stages
+(3 stages)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
         <v>1028</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>270</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="7" t="n">
         <v>328</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="7" t="n">
         <v>1626</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="7" t="n">
         <v>1028</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="n">
         <v>270</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="7" t="n">
         <v>328</v>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="7" t="n">
         <v>1626</v>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="7" t="n">
+        <v>4523</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>3598</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>270</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>328</v>
+      </c>
+      <c r="N6" s="7" t="inlineStr">
         <is>
           <t>1.0×</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Note:</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>• Detection counts FULL IMAGES (one image = one data point)</t>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>• Detection counts FULL IMAGES, Classification counts BOUNDING BOX CROPS</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>• Classification counts BOUNDING BOX CROPS (one image can contain multiple boxes)</t>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>• Split performed at IMAGE level (60/20/20) → same images, different data point counts</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>• Split performed at IMAGE level (60/20/20), then crops extracted → crop counts differ</t>
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>• Augmentation ONLY on train: Detection 4.4×, Classification 3.5×</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>• Augmentation: Detection 4.4× on train only, Classification 3.5× on train only</t>
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>• Val and Test remain UNAUGMENTED for unbiased evaluation</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:J1"/>
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="A11:J11"/>
+  <mergeCells count="10">
+    <mergeCell ref="A9:N9"/>
+    <mergeCell ref="A8:N8"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A11:N11"/>
+    <mergeCell ref="A10:N10"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📐 TABLE1: Increase row heights for better text visibility
- Header rows: 35 pt (for wrapped text)
- Data rows: 30 pt (for dataset names)
- Note rows: 18 pt (standard)

User feedback: Row heights too small, text terpotong
</commit_message>
<xml_diff>
--- a/luaran/templates/tables/Table1_Dataset_Augmentation.xlsx
+++ b/luaran/templates/tables/Table1_Dataset_Augmentation.xlsx
@@ -75,7 +75,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -89,11 +89,60 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -116,6 +165,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -500,7 +552,7 @@
     <col width="8" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset</t>
@@ -511,33 +563,33 @@
           <t>Detection (Full Images)</t>
         </is>
       </c>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="11" t="n"/>
       <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Classification (Bounding Box Crops)</t>
         </is>
       </c>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
-      <c r="I1" s="3" t="n"/>
+      <c r="G1" s="10" t="n"/>
+      <c r="H1" s="10" t="n"/>
+      <c r="I1" s="11" t="n"/>
       <c r="J1" s="2" t="inlineStr">
         <is>
           <t>After Augmentation (Train Only)</t>
         </is>
       </c>
-      <c r="K1" s="3" t="n"/>
-      <c r="L1" s="3" t="n"/>
-      <c r="M1" s="3" t="n"/>
+      <c r="K1" s="10" t="n"/>
+      <c r="L1" s="10" t="n"/>
+      <c r="M1" s="11" t="n"/>
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Boxes per Image</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="n"/>
+    <row r="2" ht="35" customHeight="1">
+      <c r="A2" s="12" t="n"/>
       <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Train</t>
@@ -598,9 +650,9 @@
           <t>Test (same)</t>
         </is>
       </c>
-      <c r="N2" s="3" t="n"/>
-    </row>
-    <row r="3">
+      <c r="N2" s="12" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>IML Lifecycle
@@ -649,7 +701,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>MP-IDB Species
@@ -698,7 +750,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>MP-IDB Stages
@@ -747,7 +799,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>MD_2019 Stages
@@ -796,35 +848,35 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="18" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Note:</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
           <t>• Detection counts FULL IMAGES, Classification counts BOUNDING BOX CROPS</t>
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
           <t>• Split performed at IMAGE level (60/20/20) → same images, different data point counts</t>
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
           <t>• Augmentation ONLY on train: Detection 4.4×, Classification 3.5×</t>
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="18" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
           <t>• Val and Test remain UNAUGMENTED for unbiased evaluation</t>

</xml_diff>